<commit_message>
fix(affiliate): resolve profile page rendering and race condition across roles and tiers
</commit_message>
<xml_diff>
--- a/docs/files-completion-list/ui-pages-trading-alerts-saas-public-testing-results.xlsx
+++ b/docs/files-completion-list/ui-pages-trading-alerts-saas-public-testing-results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SaaS Project\trading-alerts-saas-public\docs\files-completion-list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71618209-5C09-4A5E-A323-AD9A533CBBEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E51490C-3053-41A0-AC81-040E2B2CA275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" xr2:uid="{226B384D-6115-4E82-9FF4-20CA6CB65055}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1622" uniqueCount="875">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1623" uniqueCount="879">
   <si>
     <t xml:space="preserve"> Index </t>
   </si>
@@ -2617,12 +2617,6 @@
     <t>System Status (working incorrectly)</t>
   </si>
   <si>
-    <t>Should remove button (in the UI) to bar user from accessing this page (Just Implementing UI modification)</t>
-  </si>
-  <si>
-    <t>This page is redundancy with index 76 and should remove button (in the UI) to bar user from accessing it (Just Implement UI modification)</t>
-  </si>
-  <si>
     <t>Proposed Modification for FREE user account</t>
   </si>
   <si>
@@ -2635,38 +2629,56 @@
     <t>Proposed Modification for AFFILIATE+FREE user account</t>
   </si>
   <si>
-    <t>It should redirect to page that inform user "You are Already a AFFILIATE Member"</t>
-  </si>
-  <si>
-    <t>Affiliate Profile page should be displayed instead of showing Something went wrong</t>
-  </si>
-  <si>
     <t>Proposed Modification for AFFILIATE+PRO user account</t>
   </si>
   <si>
-    <t>It should display Payout Settings page as the same as AFFILIATE+FREE user account instead of showing Become an Affiliate</t>
-  </si>
-  <si>
     <t>Choose Your Plan (working incorrectly)</t>
   </si>
   <si>
-    <t>Make it redirect to "You are Already a PRO Member" page as similar to checkout page</t>
-  </si>
-  <si>
     <t>Proposed Modification for ADMIN+PRO user account</t>
   </si>
   <si>
-    <t>Make it redicrec to Admn executive dashboard</t>
-  </si>
-  <si>
-    <t>Make it redirect to Sign in Page</t>
+    <t>Resolved by redirect to Sign in Page</t>
+  </si>
+  <si>
+    <t>Resolved : URL and button in navigating to Settings - System Status was removed</t>
+  </si>
+  <si>
+    <t>Resolved : Now this page is "You are Already a PRO Member"</t>
+  </si>
+  <si>
+    <t>Resolved : It is currently redirected to "You are Already a AFFILIATE Member"</t>
+  </si>
+  <si>
+    <t>Resolved : It is currently redirected to Terms of Service Page</t>
+  </si>
+  <si>
+    <t>Resolved : It is currently redirected to Payout History Page</t>
+  </si>
+  <si>
+    <t>Resolved : It is currently redirected to You are Already an Affiliate Partner</t>
+  </si>
+  <si>
+    <t>Resolved : It is currently redirected to You are Already a PRO Member</t>
+  </si>
+  <si>
+    <t>Resolved : It is currently redirected to You are Already a PRO Member page</t>
+  </si>
+  <si>
+    <t>Resolved : it is currently redirected to Admin executive dashboard</t>
+  </si>
+  <si>
+    <t>UNRESOLVED : Affiliate Profile page should be displayed instead of showing Something went wrong</t>
+  </si>
+  <si>
+    <t>UNRESOVED : Affiliate Profile page should be displayed instead of showing Something went wrong</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2742,8 +2754,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2792,6 +2811,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -2806,7 +2831,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -2844,6 +2869,7 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3165,11 +3191,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B21EDD11-0712-4E9B-9D43-4012822F0DE1}">
-  <dimension ref="A1:AE93"/>
+  <dimension ref="A1:W93"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="7.3125" customWidth="1"/>
-    <col min="2" max="2" width="8.83984375" customWidth="1"/>
+    <col min="1" max="1" width="7.3125" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="8.83984375" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="37.62890625" customWidth="1"/>
     <col min="4" max="4" width="38.7890625" customWidth="1"/>
     <col min="5" max="5" width="23.05078125" customWidth="1"/>
@@ -3180,11 +3206,13 @@
     <col min="10" max="10" width="82" customWidth="1"/>
     <col min="11" max="11" width="13.83984375" customWidth="1"/>
     <col min="12" max="12" width="41.3125" customWidth="1"/>
-    <col min="13" max="13" width="93.20703125" customWidth="1"/>
+    <col min="13" max="13" width="21.89453125" customWidth="1"/>
     <col min="14" max="15" width="39.7890625" customWidth="1"/>
     <col min="16" max="17" width="39.41796875" customWidth="1"/>
-    <col min="18" max="19" width="40.734375" customWidth="1"/>
-    <col min="20" max="21" width="39.26171875" customWidth="1"/>
+    <col min="18" max="18" width="32.5234375" customWidth="1"/>
+    <col min="19" max="19" width="63.41796875" customWidth="1"/>
+    <col min="20" max="20" width="39.26171875" customWidth="1"/>
+    <col min="21" max="21" width="52.26171875" customWidth="1"/>
     <col min="22" max="23" width="57.47265625" customWidth="1"/>
     <col min="24" max="26" width="8.83984375" customWidth="1"/>
   </cols>
@@ -3233,31 +3261,31 @@
         <v>809</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="P1" s="6" t="s">
         <v>810</v>
       </c>
       <c r="Q1" s="6" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="R1" s="6" t="s">
         <v>827</v>
       </c>
       <c r="S1" s="6" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="T1" s="6" t="s">
         <v>828</v>
       </c>
       <c r="U1" s="6" t="s">
-        <v>868</v>
+        <v>864</v>
       </c>
       <c r="V1" s="6" t="s">
         <v>829</v>
       </c>
       <c r="W1" s="6" t="s">
-        <v>872</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.55000000000000004">
@@ -5363,7 +5391,7 @@
         <v>825</v>
       </c>
       <c r="M37" s="11" t="s">
-        <v>874</v>
+        <v>867</v>
       </c>
       <c r="N37" s="15" t="s">
         <v>760</v>
@@ -5385,7 +5413,7 @@
         <v>821</v>
       </c>
       <c r="W37" s="26" t="s">
-        <v>873</v>
+        <v>876</v>
       </c>
     </row>
     <row r="38" spans="1:23" x14ac:dyDescent="0.55000000000000004">
@@ -5426,7 +5454,7 @@
         <v>825</v>
       </c>
       <c r="M38" s="11" t="s">
-        <v>874</v>
+        <v>867</v>
       </c>
       <c r="N38" s="15" t="s">
         <v>760</v>
@@ -5448,7 +5476,7 @@
         <v>821</v>
       </c>
       <c r="W38" s="26" t="s">
-        <v>873</v>
+        <v>876</v>
       </c>
     </row>
     <row r="39" spans="1:23" x14ac:dyDescent="0.55000000000000004">
@@ -5489,7 +5517,7 @@
         <v>825</v>
       </c>
       <c r="M39" s="11" t="s">
-        <v>874</v>
+        <v>867</v>
       </c>
       <c r="N39" s="15" t="s">
         <v>760</v>
@@ -5511,7 +5539,7 @@
         <v>821</v>
       </c>
       <c r="W39" s="26" t="s">
-        <v>873</v>
+        <v>876</v>
       </c>
     </row>
     <row r="40" spans="1:23" x14ac:dyDescent="0.55000000000000004">
@@ -5552,7 +5580,7 @@
         <v>825</v>
       </c>
       <c r="M40" s="11" t="s">
-        <v>874</v>
+        <v>867</v>
       </c>
       <c r="N40" s="15" t="s">
         <v>760</v>
@@ -5570,13 +5598,13 @@
         <v>821</v>
       </c>
       <c r="U40" s="30" t="s">
-        <v>869</v>
+        <v>872</v>
       </c>
       <c r="V40" s="26" t="s">
         <v>821</v>
       </c>
       <c r="W40" s="26" t="s">
-        <v>873</v>
+        <v>876</v>
       </c>
     </row>
     <row r="41" spans="1:23" x14ac:dyDescent="0.55000000000000004">
@@ -5617,7 +5645,7 @@
         <v>825</v>
       </c>
       <c r="M41" s="11" t="s">
-        <v>874</v>
+        <v>867</v>
       </c>
       <c r="N41" s="15" t="s">
         <v>760</v>
@@ -5639,7 +5667,7 @@
         <v>821</v>
       </c>
       <c r="W41" s="26" t="s">
-        <v>873</v>
+        <v>876</v>
       </c>
     </row>
     <row r="42" spans="1:23" x14ac:dyDescent="0.55000000000000004">
@@ -5680,7 +5708,7 @@
         <v>825</v>
       </c>
       <c r="M42" s="11" t="s">
-        <v>874</v>
+        <v>867</v>
       </c>
       <c r="N42" s="15" t="s">
         <v>760</v>
@@ -5693,18 +5721,20 @@
       <c r="R42" s="23" t="s">
         <v>820</v>
       </c>
-      <c r="S42" s="23" t="s">
-        <v>867</v>
+      <c r="S42" s="31" t="s">
+        <v>877</v>
       </c>
       <c r="T42" s="28" t="s">
         <v>826</v>
       </c>
-      <c r="U42" s="28"/>
+      <c r="U42" s="31" t="s">
+        <v>878</v>
+      </c>
       <c r="V42" s="26" t="s">
         <v>821</v>
       </c>
       <c r="W42" s="26" t="s">
-        <v>873</v>
+        <v>876</v>
       </c>
     </row>
     <row r="43" spans="1:23" x14ac:dyDescent="0.55000000000000004">
@@ -5745,7 +5775,7 @@
         <v>825</v>
       </c>
       <c r="M43" s="11" t="s">
-        <v>874</v>
+        <v>867</v>
       </c>
       <c r="N43" s="15" t="s">
         <v>760</v>
@@ -5767,7 +5797,7 @@
         <v>821</v>
       </c>
       <c r="W43" s="26" t="s">
-        <v>873</v>
+        <v>876</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.55000000000000004">
@@ -5808,7 +5838,7 @@
         <v>825</v>
       </c>
       <c r="M44" s="11" t="s">
-        <v>874</v>
+        <v>867</v>
       </c>
       <c r="N44" s="15" t="s">
         <v>760</v>
@@ -5830,7 +5860,7 @@
         <v>821</v>
       </c>
       <c r="W44" s="26" t="s">
-        <v>873</v>
+        <v>876</v>
       </c>
     </row>
     <row r="45" spans="1:23" x14ac:dyDescent="0.55000000000000004">
@@ -5883,19 +5913,19 @@
         <v>821</v>
       </c>
       <c r="S45" s="23" t="s">
-        <v>866</v>
+        <v>870</v>
       </c>
       <c r="T45" s="30" t="s">
         <v>821</v>
       </c>
       <c r="U45" s="30" t="s">
-        <v>866</v>
+        <v>873</v>
       </c>
       <c r="V45" s="26" t="s">
         <v>821</v>
       </c>
       <c r="W45" s="26" t="s">
-        <v>873</v>
+        <v>876</v>
       </c>
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.55000000000000004">
@@ -5948,19 +5978,19 @@
         <v>821</v>
       </c>
       <c r="S46" s="23" t="s">
-        <v>866</v>
+        <v>870</v>
       </c>
       <c r="T46" s="30" t="s">
         <v>821</v>
       </c>
       <c r="U46" s="30" t="s">
-        <v>866</v>
+        <v>873</v>
       </c>
       <c r="V46" s="26" t="s">
         <v>821</v>
       </c>
       <c r="W46" s="26" t="s">
-        <v>873</v>
+        <v>876</v>
       </c>
     </row>
     <row r="47" spans="1:23" x14ac:dyDescent="0.55000000000000004">
@@ -6021,7 +6051,7 @@
         <v>822</v>
       </c>
       <c r="W47" s="26" t="s">
-        <v>873</v>
+        <v>876</v>
       </c>
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.55000000000000004">
@@ -6062,7 +6092,7 @@
         <v>825</v>
       </c>
       <c r="M48" s="11" t="s">
-        <v>874</v>
+        <v>867</v>
       </c>
       <c r="N48" s="15" t="s">
         <v>760</v>
@@ -6084,7 +6114,7 @@
         <v>821</v>
       </c>
       <c r="W48" s="26" t="s">
-        <v>873</v>
+        <v>876</v>
       </c>
     </row>
     <row r="49" spans="1:23" x14ac:dyDescent="0.55000000000000004">
@@ -6196,19 +6226,19 @@
         <v>823</v>
       </c>
       <c r="S50" s="23" t="s">
-        <v>866</v>
+        <v>870</v>
       </c>
       <c r="T50" s="30" t="s">
         <v>823</v>
       </c>
       <c r="U50" s="30" t="s">
-        <v>866</v>
+        <v>873</v>
       </c>
       <c r="V50" s="26" t="s">
         <v>823</v>
       </c>
       <c r="W50" s="26" t="s">
-        <v>873</v>
+        <v>876</v>
       </c>
     </row>
     <row r="51" spans="1:23" x14ac:dyDescent="0.55000000000000004">
@@ -7316,26 +7346,26 @@
       </c>
       <c r="O69" s="15"/>
       <c r="P69" s="19" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
       <c r="Q69" s="19" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="R69" s="21" t="s">
         <v>769</v>
       </c>
       <c r="S69" s="21"/>
       <c r="T69" s="30" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="U69" s="30" t="s">
-        <v>871</v>
+        <v>874</v>
       </c>
       <c r="V69" s="26" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="W69" s="26" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
     </row>
     <row r="70" spans="1:23" x14ac:dyDescent="0.55000000000000004">
@@ -8084,37 +8114,37 @@
         <v>858</v>
       </c>
       <c r="M82" s="11" t="s">
-        <v>861</v>
+        <v>867</v>
       </c>
       <c r="N82" s="16" t="s">
         <v>858</v>
       </c>
       <c r="O82" s="16" t="s">
-        <v>861</v>
+        <v>871</v>
       </c>
       <c r="P82" s="19" t="s">
         <v>858</v>
       </c>
       <c r="Q82" s="19" t="s">
-        <v>861</v>
+        <v>871</v>
       </c>
       <c r="R82" s="23" t="s">
         <v>858</v>
       </c>
       <c r="S82" s="23" t="s">
-        <v>861</v>
+        <v>871</v>
       </c>
       <c r="T82" s="30" t="s">
         <v>858</v>
       </c>
       <c r="U82" s="30" t="s">
-        <v>861</v>
+        <v>871</v>
       </c>
       <c r="V82" s="26" t="s">
         <v>858</v>
       </c>
       <c r="W82" s="26" t="s">
-        <v>861</v>
+        <v>871</v>
       </c>
     </row>
     <row r="83" spans="1:23" x14ac:dyDescent="0.55000000000000004">
@@ -8214,37 +8244,37 @@
         <v>859</v>
       </c>
       <c r="M84" s="11" t="s">
-        <v>860</v>
+        <v>867</v>
       </c>
       <c r="N84" s="16" t="s">
         <v>859</v>
       </c>
       <c r="O84" s="16" t="s">
-        <v>860</v>
+        <v>868</v>
       </c>
       <c r="P84" s="19" t="s">
         <v>859</v>
       </c>
       <c r="Q84" s="19" t="s">
-        <v>860</v>
+        <v>868</v>
       </c>
       <c r="R84" s="23" t="s">
         <v>859</v>
       </c>
       <c r="S84" s="23" t="s">
-        <v>860</v>
+        <v>868</v>
       </c>
       <c r="T84" s="30" t="s">
         <v>859</v>
       </c>
       <c r="U84" s="30" t="s">
-        <v>860</v>
+        <v>868</v>
       </c>
       <c r="V84" s="26" t="s">
         <v>859</v>
       </c>
       <c r="W84" s="26" t="s">
-        <v>860</v>
+        <v>868</v>
       </c>
     </row>
     <row r="85" spans="1:23" x14ac:dyDescent="0.55000000000000004">

</xml_diff>